<commit_message>
chore(imports): regenerate responsables_exemple.xlsx with a student code link
🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/docs/import-templates/responsables_exemple.xlsx
+++ b/docs/import-templates/responsables_exemple.xlsx
@@ -399,13 +399,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -424,6 +425,9 @@
       <c r="E1" t="str">
         <v>Adresse</v>
       </c>
+      <c r="F1" t="str">
+        <v>Code élève</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -441,6 +445,9 @@
       <c r="E2" t="str">
         <v>N Djamena</v>
       </c>
+      <c r="F2" t="str">
+        <v>NDS-DEMO-2026-X00001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,14 +473,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -546,62 +553,74 @@
         <v>Optionnel.</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Remarques</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Code élève</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Optionnel. Lie automatiquement le responsable à l'élève portant ce code (importé avant ou déjà présent dans l'école).</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Optionnel. Lie automatiquement le responsable à l'élève portant ce code (importé avant ou déjà présent dans l'école).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>- Ne modifiez pas la premiere ligne : elle contient les en-tetes.</v>
+        <v>Remarques</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>- Ajoutez une ligne par personne a partir de la ligne 2 ; les lignes vides sont ignorees.</v>
+        <v>- Ne modifiez pas la premiere ligne : elle contient les en-tetes.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>- Les dates s'ecrivent JJ/MM/AAAA (ex. 14/03/2012) ou AAAA-MM-JJ (ex. 2012-03-14).</v>
+        <v>- Ajoutez une ligne par personne a partir de la ligne 2 ; les lignes vides sont ignorees.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>- Sexe : M, F ou AUTRE.</v>
+        <v>- Les dates s'ecrivent JJ/MM/AAAA (ex. 14/03/2012) ou AAAA-MM-JJ (ex. 2012-03-14).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>- Code : optionnel. Laisses vide, un code est genere automatiquement.</v>
+        <v>- Sexe : M, F ou AUTRE.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>- Un code utilise deux fois dans le fichier (ou deja present dans l'ecole) est refuse.</v>
+        <v>- Code : optionnel. Laisses vide, un code est genere automatiquement.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>- Un code utilise deux fois dans le fichier (ou deja present dans l'ecole) est refuse.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>- Ligne d'exemple : voir la feuille « Exemples » (non importee).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -620,10 +639,13 @@
       <c r="E1" t="str">
         <v>Adresse</v>
       </c>
+      <c r="F1" t="str">
+        <v>Code élève</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>